<commit_message>
feat: integrate sanitized corporate layouts with conservative table binding
</commit_message>
<xml_diff>
--- a/resources/corporate_format.xlsx
+++ b/resources/corporate_format.xlsx
@@ -53214,14 +53214,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24"/>
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>DAFTAR PENYUSUTAN DAN AMORTISASI FISKAL</t>
+        </is>
+      </c>
       <c r="B1" s="24"/>
       <c r="C1" s="24"/>
       <c r="D1" s="24"/>
       <c r="E1" s="24"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A3" s="13"/>
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>HARTA BERWUJUD KELOMPOK 1</t>
+        </is>
+      </c>
     </row>
     <row r="4" spans="1:9" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="inlineStr">
@@ -55299,7 +55307,11 @@
       <c r="I188" s="1"/>
     </row>
     <row r="191" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A191" s="13"/>
+      <c r="A191" s="13" t="inlineStr">
+        <is>
+          <t>HARTA BERWUJUD KELOMPOK 2</t>
+        </is>
+      </c>
     </row>
     <row r="192" spans="1:9" s="27" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="10" t="inlineStr">
@@ -55375,7 +55387,11 @@
       <c r="I194" s="1"/>
     </row>
     <row r="197" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A197" s="13"/>
+      <c r="A197" s="13" t="inlineStr">
+        <is>
+          <t>HARTA BERWUJUD KELOMPOK 3</t>
+        </is>
+      </c>
     </row>
     <row r="198" spans="1:9" s="20" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A198" s="11" t="inlineStr">
@@ -55451,7 +55467,11 @@
       <c r="I200" s="12"/>
     </row>
     <row r="203" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A203" s="13"/>
+      <c r="A203" s="13" t="inlineStr">
+        <is>
+          <t>HARTA BERWUJUD KELOMPOK 4</t>
+        </is>
+      </c>
     </row>
     <row r="204" spans="1:9" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A204" s="11" t="inlineStr">
@@ -55607,7 +55627,11 @@
       <c r="I212" s="12"/>
     </row>
     <row r="215" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A215" s="13"/>
+      <c r="A215" s="13" t="inlineStr">
+        <is>
+          <t>BANGUNAN - PERMANEN</t>
+        </is>
+      </c>
     </row>
     <row r="216" spans="1:9" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A216" s="11" t="inlineStr">
@@ -55683,7 +55707,11 @@
       <c r="I218" s="12"/>
     </row>
     <row r="221" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A221" s="13"/>
+      <c r="A221" s="13" t="inlineStr">
+        <is>
+          <t>BANGUNAN - TIDAK PERMANEN</t>
+        </is>
+      </c>
     </row>
     <row r="222" spans="1:9" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A222" s="11" t="inlineStr">
@@ -55801,7 +55829,11 @@
       <c r="H228" s="12"/>
     </row>
     <row r="230" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A230" s="13"/>
+      <c r="A230" s="13" t="inlineStr">
+        <is>
+          <t>HARTA TIDAK BERWUJUD - KELOMPOK 1</t>
+        </is>
+      </c>
     </row>
     <row r="231" spans="1:9" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A231" s="11" t="inlineStr">
@@ -55877,7 +55909,11 @@
       <c r="I233" s="12"/>
     </row>
     <row r="236" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A236" s="13"/>
+      <c r="A236" s="13" t="inlineStr">
+        <is>
+          <t>HARTA TIDAK BERWUJUD - KELOMPOK 2</t>
+        </is>
+      </c>
     </row>
     <row r="237" spans="1:9" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A237" s="11" t="inlineStr">
@@ -55953,7 +55989,11 @@
       <c r="I239" s="12"/>
     </row>
     <row r="242" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A242" s="13"/>
+      <c r="A242" s="13" t="inlineStr">
+        <is>
+          <t>HARTA TIDAK BERWUJUD - KELOMPOK 3</t>
+        </is>
+      </c>
     </row>
     <row r="243" spans="1:9" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A243" s="11" t="inlineStr">
@@ -56029,7 +56069,11 @@
       <c r="I245" s="12"/>
     </row>
     <row r="248" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A248" s="13"/>
+      <c r="A248" s="13" t="inlineStr">
+        <is>
+          <t>HARTA TIDAK BERWUJUD - KELOMPOK 4</t>
+        </is>
+      </c>
     </row>
     <row r="249" spans="1:9" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A249" s="11" t="inlineStr">
@@ -56105,7 +56149,11 @@
       <c r="I251" s="17"/>
     </row>
     <row r="254" spans="1:9" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A254" s="13"/>
+      <c r="A254" s="13" t="inlineStr">
+        <is>
+          <t>HARTA TIDAK BERWUJUD - KELOMPOK LAINNYA</t>
+        </is>
+      </c>
     </row>
     <row r="255" spans="1:9" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A255" s="11" t="inlineStr">

</xml_diff>

<commit_message>
feat: bind corporate asset groups and numeric scalar fields
</commit_message>
<xml_diff>
--- a/resources/corporate_format.xlsx
+++ b/resources/corporate_format.xlsx
@@ -484,7 +484,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13"/>
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>DALAM HAL WAJIB PAJAK DALAM TAHUN PAJAK INI MELAKUKAN TRANSAKSI DENGAN PIHAK-PIHAK YANG MERUPAKAN PENDUDUK TAX HAVEN COUNTRY</t>
+        </is>
+      </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="inlineStr">
@@ -537,13 +541,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="28"/>
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>RINCIAN BIAYA TERTENTU</t>
+        </is>
+      </c>
       <c r="B1" s="28"/>
       <c r="C1" s="28"/>
       <c r="D1" s="28"/>
     </row>
     <row r="2" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> I. DAFTAR NOMINATIF BIAYA PROMOSI DAN PENJUALAN, SERTA PENGGANTIAN ATAU IMBALAN DALAM BENTUK NATURA DAN/ATAU KENIKMATAN </t>
+        </is>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="inlineStr">
@@ -610,7 +622,11 @@
       <c r="J4" s="1"/>
     </row>
     <row r="6" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13"/>
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> II. DAFTAR NOMINATIF BIAYA ENTERTAINMENT </t>
+        </is>
+      </c>
     </row>
     <row r="7" spans="1:10" s="13" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="inlineStr">
@@ -4085,7 +4101,11 @@
       <c r="J292" s="1"/>
     </row>
     <row r="295" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A295" s="13"/>
+      <c r="A295" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> III. DAFTAR PIUTANG YANG NYATA-NYATA TIDAK DAPAT DITAGIH </t>
+        </is>
+      </c>
     </row>
     <row r="296" spans="1:10" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A296" s="11" t="inlineStr">
@@ -4142,7 +4162,11 @@
       <c r="I297" s="1"/>
     </row>
     <row r="299" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A299" s="13"/>
+      <c r="A299" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> IV. RINCIAN BAGI WAJIB PAJAK PEMBERI NATURA DAN/ATAU KENIKMATAN - DAFTAR SARANA DAN FASILITAS SERTA PENYUSUTANNYA </t>
+        </is>
+      </c>
     </row>
     <row r="300" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A300" s="11" t="inlineStr">
@@ -4191,7 +4215,11 @@
       <c r="G301" s="11"/>
     </row>
     <row r="303" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A303" s="13"/>
+      <c r="A303" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> V. DAFTAR DEBITUR NON-PERFORMING LOAN </t>
+        </is>
+      </c>
     </row>
     <row r="304" spans="1:10" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A304" s="10" t="inlineStr">
@@ -4268,7 +4296,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13"/>
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> I. PERHITUNGAN EBITDA </t>
+        </is>
+      </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="inlineStr">
@@ -4319,7 +4351,11 @@
       <c r="B7" s="1"/>
     </row>
     <row r="10" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13"/>
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> II. PERBANDINGAN ANTARA UTANG DAN MODAL (DEBT TO EQUITY RATIO) - PENGHITUNGAN RATA-RATA SALDO UTANG </t>
+        </is>
+      </c>
     </row>
     <row r="11" spans="1:16" s="20" customFormat="1" ht="78" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="inlineStr">
@@ -4444,7 +4480,11 @@
       <c r="P13" s="12"/>
     </row>
     <row r="16" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="13"/>
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> II. PERBANDINGAN ANTARA UTANG DAN MODAL (DEBT TO EQUITY RATIO) - PENGHITUNGAN SALDO RATA-RATA MODAL </t>
+        </is>
+      </c>
     </row>
     <row r="17" spans="1:14" s="20" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="inlineStr">
@@ -4634,7 +4674,11 @@
       <c r="D27" s="34"/>
     </row>
     <row r="29" spans="1:14" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="13"/>
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> III. PENGHITUNGAN BIAYA PINJAMAN </t>
+        </is>
+      </c>
     </row>
     <row r="30" spans="1:14" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="inlineStr">
@@ -4712,7 +4756,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13"/>
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> LAPORAN UTANG SWASTA LUAR NEGERI </t>
+        </is>
+      </c>
     </row>
     <row r="2" spans="1:16" s="20" customFormat="1" ht="72" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="inlineStr">
@@ -4859,8 +4907,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14"/>
-      <c r="B1" s="14"/>
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Nilai sumber</t>
+        </is>
+      </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="inlineStr">
@@ -5715,7 +5771,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13"/>
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> A. DAFTAR PEMEGANG SAHAM/PEMILIK MODAL DAN JUMLAH DIVIDEN/PEMBAGIAN LABA YANG DIBAGIKAN SERTA DAFTAR SUSUNAN PENGURUS DAN KOMISARIS </t>
+        </is>
+      </c>
     </row>
     <row r="2" spans="1:12" s="19" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="inlineStr">
@@ -5846,7 +5906,11 @@
       <c r="I9" s="12"/>
     </row>
     <row r="11" spans="1:12" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="13"/>
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> B. DAFTAR PENYERTAAN MODAL, UTANG, DAN/ATAU PIUTANG PADA PERUSAHAAN AFILIASI </t>
+        </is>
+      </c>
     </row>
     <row r="12" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="inlineStr">
@@ -52807,7 +52871,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13"/>
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> A. PENGHASILAN YANG DIKENAKAN PPh YANG BERSIFAT FINAL </t>
+        </is>
+      </c>
     </row>
     <row r="2" spans="1:7" s="20" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="inlineStr">
@@ -52869,7 +52937,11 @@
       <c r="G4" s="1"/>
     </row>
     <row r="7" spans="1:7" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="13"/>
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> B. PENGHASILAN YANG TIDAK TERMASUK OBJEK PAJAK </t>
+        </is>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="inlineStr">
@@ -52939,7 +53011,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8"/>
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>ANGSURAN PAJAK PENGHASILAN TAHUN PAJAK BERJALAN</t>
+        </is>
+      </c>
       <c r="B1" s="8"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>